<commit_message>
docs(ltssm): regenerate workbook with the width and scrambling findings
Catches docs/ltssm.xlsx up to the generator; the file had been locked by an open
spreadsheet across the last two commits. Findings now 17 rows: 14 rewritten with
the narrow-partner reproducer, 15 splitting out Lane reversal, and 16/17 covering
the missing scrambler and the absent MAC packet datapath.
</commit_message>
<xml_diff>
--- a/docs/ltssm.xlsx
+++ b/docs/ltssm.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes (holds here)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -234,7 +234,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -301,7 +301,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -435,7 +435,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -502,7 +502,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes (Idle only, no DLL traffic)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Partial: sends TS1, timeout -&gt; Detect</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1 blocker</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Adapter output, not yet consumed</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -3003,7 +3003,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
     </row>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -3040,7 +3040,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1 blocker</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -3077,7 +3077,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1 blocker</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
@@ -3099,7 +3099,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -3114,167 +3114,167 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rxstatus_skp_add_i / _rem_i</t>
+          <t xml:space="preserve">rx_err_i</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LANES each</t>
+          <t xml:space="preserve">1 (link-level OR)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pipe adapter decode</t>
+          <t xml:space="preserve">os_rx rxstatus decode</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L0</t>
+          <t xml:space="preserve">L0 -&gt; Recovery</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SKP added/removed (expected, not an error)</t>
+          <t xml:space="preserve">Decode (100), EB overflow/underflow (101/110) and disparity (111) errors; SKP add/remove are not errors</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">Done (per-Lane reporting still M2)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rxstatus_decode_err_i</t>
+          <t xml:space="preserve">ts1_pad_all_i / _any_i</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LANES</t>
+          <t xml:space="preserve">1 each</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pipe adapter decode</t>
+          <t xml:space="preserve">os_rx</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L0 -&gt; Recovery</t>
+          <t xml:space="preserve">Polling.Active</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8b/10b decode error (rxstatus=100)</t>
+          <t xml:space="preserve">8 consecutive TS1 with Link and Lane = PAD, reduced over enabled Lanes</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rxstatus_eb_over_i / _under_i</t>
+          <t xml:space="preserve">ts2_pad_all_i / _any_i</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LANES each</t>
+          <t xml:space="preserve">1 each</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pipe adapter decode</t>
+          <t xml:space="preserve">os_rx</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L0 -&gt; Recovery</t>
+          <t xml:space="preserve">Polling.Configuration</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elastic buffer overflow/underflow (101/110)</t>
+          <t xml:space="preserve">8 consecutive TS2 with Link and Lane = PAD</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rxstatus_disparity_err_i</t>
+          <t xml:space="preserve">ts1_link_all_i / _any_i</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LANES</t>
+          <t xml:space="preserve">1 each</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pipe adapter decode</t>
+          <t xml:space="preserve">os_rx</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">L0 -&gt; Recovery</t>
+          <t xml:space="preserve">Configuration.Linkwidth.Start</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disparity error (rxstatus=111)</t>
+          <t xml:space="preserve">2 consecutive TS1 with non-PAD Link and PAD Lane</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ts1_rx_valid_i / ts2_rx_valid_i</t>
+          <t xml:space="preserve">ts1_lane_all_i / _any_i</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LANES each</t>
+          <t xml:space="preserve">1 each</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -3284,34 +3284,34 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Partial: 1 bit, tied 0</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Polling, Configuration</t>
+          <t xml:space="preserve">Configuration.Linkwidth.Accept, Lanenum.Wait/Accept</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Per-Lane TS reception (currently a single link-wide bit)</t>
+          <t xml:space="preserve">2 consecutive TS1 with non-PAD Link and Lane</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1 (widen)</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ts_rx_consec_cnt_i</t>
+          <t xml:space="preserve">ts2_cfg_all_i / _any_i</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4+ bits per Lane</t>
+          <t xml:space="preserve">1 each</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -3321,34 +3321,34 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Polling (8 consecutive), Configuration (2 consecutive), Config.Complete (8)</t>
+          <t xml:space="preserve">Configuration.Complete</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consecutive matching-TS counters - the actual exit criteria</t>
+          <t xml:space="preserve">8 consecutive TS2 with non-PAD Link and Lane</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1 blocker</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ts_rx_link_num_i</t>
+          <t xml:space="preserve">idle_all_i / _any_i</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 x LANES</t>
+          <t xml:space="preserve">1 each</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3358,34 +3358,34 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Config.Linkwidth.*</t>
+          <t xml:space="preserve">Config.Idle, Recovery.Idle</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Received Link number</t>
+          <t xml:space="preserve">8 consecutive Idle Symbol Times; counted as non-K Symbol Times so it holds whether or not the PHY scrambles</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done (revisit if a MAC scrambler lands)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ts_rx_lane_num_i</t>
+          <t xml:space="preserve">rx_link_num_i</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 x LANES</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3395,34 +3395,34 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Config.Lanenum.*</t>
+          <t xml:space="preserve">Config.Linkwidth.*</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Received Lane number</t>
+          <t xml:space="preserve">Received Link number</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ts_rx_link_is_pad_i / lane_is_pad_i</t>
+          <t xml:space="preserve">rx_lane_num_i</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LANES each</t>
+          <t xml:space="preserve">8 x LANES</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -3432,34 +3432,34 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Polling, Configuration</t>
+          <t xml:space="preserve">Config.Lanenum.*</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAD (K23.7) detection - drives most Config decisions</t>
+          <t xml:space="preserve">Received Lane numbers, compared against what we transmit</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ts_rx_lane_num_changed_i</t>
+          <t xml:space="preserve">rx_lane_num_changed_i</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LANES</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">os_rx drives it; LTSSM uses a match compare instead</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -3484,19 +3484,19 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ts_rx_rate_id_i</t>
+          <t xml:space="preserve">rx_rate_id_i</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 x LANES</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -3516,24 +3516,24 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Remote advertised data rates; recorded for later speed change</t>
+          <t xml:space="preserve">Remote advertised data rates; recorded for the later speed change</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ts_rx_n_fts_i</t>
+          <t xml:space="preserve">rx_n_fts_i</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 x LANES</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -3553,24 +3553,24 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N_FTS must be noted when leaving Config.Complete</t>
+          <t xml:space="preserve">N_FTS noted when leaving Config.Complete</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">Done (used by L0s later)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ts_rx_training_ctrl_i</t>
+          <t xml:space="preserve">rx_train_ctrl_i</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 x LANES</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Captured in os_rx, not routed to the LTSSM</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -3632,19 +3632,19 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">idle_rx_consec_i</t>
+          <t xml:space="preserve">deskew_done_i</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">count per Lane</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3654,113 +3654,113 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes (simplified)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Config.Idle, Recovery.Idle</t>
+          <t xml:space="preserve">Config.Complete exit</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consecutive Idle data Symbol Times received (8 required)</t>
+          <t xml:space="preserve">Lane-to-Lane de-skew complete; today only checks that every enabled Lane saw a TS in the same cycle</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">M3 (real skew correction)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">deskew_done_i</t>
+          <t xml:space="preserve">os_sent_cnt_i</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">12</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_rx</t>
+          <t xml:space="preserve">os_tx</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Config.Complete exit</t>
+          <t xml:space="preserve">Polling.Active (1024 TS1), Polling.Config (16 TS2), Config.Complete (16 TS2), Config.Idle (16 Idle Symbols)</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lane-to-Lane de-skew complete (mandatory on exit)</t>
+          <t xml:space="preserve">Ordered sets sent since os_cnt_clr; Idle counts Symbols instead of sets</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1 (x2/x4)</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ts_tx_count_i</t>
+          <t xml:space="preserve">timer_expired (internal)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">11+ bits</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx</t>
+          <t xml:space="preserve">rivet_mac_timer</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Polling.Active (1024 TS1), Polling.Config (16 TS2), Config.Complete (16 TS2)</t>
+          <t xml:space="preserve">Detect.Quiet, Detect.Active retry, Polling.*, Configuration.*, Recovery.*</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transmitted ordered-set counters</t>
+          <t xml:space="preserve">12 / 24 / 48 / 2 ms timeouts, divided by LTSSM_TIMER_SCALE for simulation</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1 blocker</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">idle_tx_count_i</t>
+          <t xml:space="preserve">cfg_link_training_enable_i</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5+ bits</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx</t>
+          <t xml:space="preserve">TL / config space</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -3770,34 +3770,34 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Config.Idle (16 Idle Symbols)</t>
+          <t xml:space="preserve">leaving Detect</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transmitted Idle Symbol counter</t>
+          <t xml:space="preserve">PG213 cfg_link_training_enable gate</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx_busy_i / done_i</t>
+          <t xml:space="preserve">cfg_link_disable_i</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 each</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx</t>
+          <t xml:space="preserve">TL / config space</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -3807,34 +3807,34 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">all TX states</t>
+          <t xml:space="preserve">Disabled</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handshake that a requested OS burst is in flight / finished</t>
+          <t xml:space="preserve">Link Disable bit</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Later</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">timer_expired_i</t>
+          <t xml:space="preserve">cfg_retrain_link_i</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 (or per-timer)</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivet_mac_timer (new)</t>
+          <t xml:space="preserve">TL / config space</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3844,24 +3844,24 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detect.Quiet, Polling.*, Configuration.*, Recovery.*</t>
+          <t xml:space="preserve">Recovery entry</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 / 24 / 48 / 2 ms timeouts; sim-abbreviated by parameter</t>
+          <t xml:space="preserve">Retrain Link bit (Link Control)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1 blocker</t>
+          <t xml:space="preserve">Later</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cfg_link_training_enable_i</t>
+          <t xml:space="preserve">cfg_enter_compliance_i</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -3881,29 +3881,29 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">leaving Detect</t>
+          <t xml:space="preserve">Polling.Compliance</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PG213 cfg_link_training_enable gate</t>
+          <t xml:space="preserve">Link Control 2 bit 4</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">Later</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cfg_link_disable_i</t>
+          <t xml:space="preserve">cfg_target_link_speed_i</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -3918,24 +3918,24 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disabled</t>
+          <t xml:space="preserve">Recovery.Speed</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Link Disable bit</t>
+          <t xml:space="preserve">Target Link Speed (Link Control 2)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">M4</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cfg_retrain_link_i</t>
+          <t xml:space="preserve">cfg_select_deemphasis_i</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -3955,24 +3955,24 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recovery entry</t>
+          <t xml:space="preserve">Detect.Quiet, Gen2 de-emphasis</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retrain Link bit (Link Control)</t>
+          <t xml:space="preserve">select_deemphasis variable / Link Control 2</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">M4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cfg_enter_compliance_i</t>
+          <t xml:space="preserve">cfg_hot_reset_i</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3992,12 +3992,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Polling.Compliance</t>
+          <t xml:space="preserve">Hot_Reset</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Link Control 2 bit 4</t>
+          <t xml:space="preserve">Secondary bus reset propagation</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -4009,44 +4009,44 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cfg_target_link_speed_i</t>
+          <t xml:space="preserve">dll_replay_timer_expired_i</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TL / config space</t>
+          <t xml:space="preserve">DLL sideband</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">In struct, not an LTSSM port</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recovery.Speed</t>
+          <t xml:space="preserve">Recovery policy</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Target Link Speed (Link Control 2)</t>
+          <t xml:space="preserve">REPLAY_NUM rollover hint</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M4</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cfg_select_deemphasis_i</t>
+          <t xml:space="preserve">dll_nak_storm_i</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -4056,34 +4056,34 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TL / config space</t>
+          <t xml:space="preserve">DLL sideband</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">In struct, not an LTSSM port</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detect.Quiet, Gen2 de-emphasis</t>
+          <t xml:space="preserve">Recovery policy</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">select_deemphasis variable / Link Control 2</t>
+          <t xml:space="preserve">Excessive NAK indication</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M4</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cfg_hot_reset_i</t>
+          <t xml:space="preserve">dll_tx_idle_req_i</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -4093,136 +4093,25 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TL / config space</t>
+          <t xml:space="preserve">DLL sideband</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">In struct, not an LTSSM port</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hot_Reset</t>
+          <t xml:space="preserve">L0s / L1 entry</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Secondary bus reset propagation</t>
+          <t xml:space="preserve">DLL requests transmitter idle</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Later</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dll_replay_timer_expired_i</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLL sideband</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In struct, not an LTSSM port</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recovery policy</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">REPLAY_NUM rollover hint</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M2</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dll_nak_storm_i</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLL sideband</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In struct, not an LTSSM port</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recovery policy</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Excessive NAK indication</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M2</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dll_tx_idle_req_i</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLL sideband</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In struct, not an LTSSM port</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L0s / L1 entry</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DLL requests transmitter idle</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Later</t>
         </is>
@@ -4294,17 +4183,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes (0)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Receiver detection request (with P1 + TxElecIdle)</t>
+          <t xml:space="preserve">Receiver detection request (with P1 + TxElecIdle) in Detect.Active</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
@@ -4326,17 +4215,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes ('1)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrical Idle control per Lane</t>
+          <t xml:space="preserve">Electrical Idle through Detect and on unused Lanes</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
@@ -4358,17 +4247,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes (P1)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P0 / P0s / P1 / P2 selection</t>
+          <t xml:space="preserve">P1 in Detect, P0 elsewhere; P0s/P2 arrive with power management</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
@@ -4390,17 +4279,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes - HARDCODED Gen2 (3'd1)</t>
+          <t xml:space="preserve">Yes - 2.5 GT/s (3'd0)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MUST be 2.5 GT/s (0) for Detect..L0; Gen2 only after Recovery.Speed</t>
+          <t xml:space="preserve">2.5 GT/s for Detect..L0; Gen2 only after Recovery.Speed</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIX in M1</t>
+          <t xml:space="preserve">Done (stateful in M4)</t>
         </is>
       </c>
     </row>
@@ -4513,22 +4402,22 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivet_mac -&gt; ctrl</t>
+          <t xml:space="preserve">rivet_mac -&gt; ctrl -&gt; cfg_ltssm_state</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes, but swallowed in ctrl</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PG213 cfg_ltssm_state[5:0]; must become a controller top-level port</t>
+          <t xml:space="preserve">PG213 cfg_ltssm_state[5:0], now a port on rivet_pcie_ctrl and rivet_pcie</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
@@ -4550,17 +4439,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes (constant 0)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LinkUp: spec sets it in Configuration.Idle, not on L0 entry</t>
+          <t xml:space="preserve">LinkUp asserted in Configuration.Idle, cleared in Detect.Quiet</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
@@ -4582,17 +4471,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes (NONE)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ordered-set type request (TS1/TS2/SKP/EIOS/FTS)</t>
+          <t xml:space="preserve">Ordered-set type request (TS1/TS2/SKP/EIOS/FTS/Idle)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4503,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes (0)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -4624,19 +4513,19 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx_link_num_o</t>
+          <t xml:space="preserve">os_cnt_clr_o</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -4646,61 +4535,61 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Link number to transmit in TS</t>
+          <t xml:space="preserve">Restart the sent counter on state entry, and hold it clear until the gating ordered set has been received</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx_lane_num_o</t>
+          <t xml:space="preserve">capture_clr_o</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 x LANES</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx</t>
+          <t xml:space="preserve">os_rx</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Per-Lane Lane number to transmit</t>
+          <t xml:space="preserve">Restart the consecutive counters and field capture on state entry</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx_link_pad_o / lane_pad_o</t>
+          <t xml:space="preserve">tx_link_num_o</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 / LANES</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -4710,29 +4599,29 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Send PAD (K23.7) instead of a number</t>
+          <t xml:space="preserve">Link number to transmit in TS</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx_lane_mask_o</t>
+          <t xml:space="preserve">tx_lane_num_o</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LANES</t>
+          <t xml:space="preserve">8 x LANES</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -4742,29 +4631,29 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Which Lanes transmit the requested OS</t>
+          <t xml:space="preserve">Per-Lane Lane number to transmit; sequential 0..n-1, no reversal</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1 (x2/x4)</t>
+          <t xml:space="preserve">Done (M3: reversal)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx_rate_id_o</t>
+          <t xml:space="preserve">tx_link_pad_o / tx_lane_pad_o</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">1 each</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -4774,61 +4663,61 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Advertised data rates in TS (Gen1+Gen2 even while training at 2.5 GT/s)</t>
+          <t xml:space="preserve">Send PAD (K23.7) instead of a number</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx_n_fts_o</t>
+          <t xml:space="preserve">lane_en_o</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">LANES</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx</t>
+          <t xml:space="preserve">os_tx / os_rx</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N_FTS advertised in TS</t>
+          <t xml:space="preserve">Lanes that form the configured Link; also the reduction mask in os_rx</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx_training_ctrl_o</t>
+          <t xml:space="preserve">tx_rate_id_o</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -4838,29 +4727,29 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hot Reset / Disable Link / Loopback / Disable Scrambling / Compliance Receive</t>
+          <t xml:space="preserve">Advertised data rates in TS (2.5 + 5.0 GT/s while training at 2.5)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx_count_req_o</t>
+          <t xml:space="preserve">tx_n_fts_o</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -4870,56 +4759,56 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">How many OS to send (1024 TS1, 16 TS2, 16 Idle)</t>
+          <t xml:space="preserve">N_FTS advertised in TS (N_FTS_ADV parameter)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rxpolarity_o</t>
+          <t xml:space="preserve">tx_train_ctrl_o</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LANES</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pipe adapter -&gt; PIPE</t>
+          <t xml:space="preserve">os_tx</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO (adapter ties 0)</t>
+          <t xml:space="preserve">Yes (constant 0)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Polarity inversion request; decided in Polling.Configuration</t>
+          <t xml:space="preserve">Hot Reset / Disable Link / Loopback / Disable Scrambling / Compliance Receive</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Later</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">txcompliance_o</t>
+          <t xml:space="preserve">rxpolarity_o</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -4934,29 +4823,29 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO (adapter ties 0)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compliance pattern control</t>
+          <t xml:space="preserve">Polarity inversion request; decided in Polling.Configuration</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">txdeemph_o</t>
+          <t xml:space="preserve">txcompliance_o</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">LANES</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -4966,61 +4855,61 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO (adapter hardcodes 1)</t>
+          <t xml:space="preserve">NO (adapter ties 0)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gen2 de-emphasis selection (-3.5 / -6 dB); negotiated, not constant</t>
+          <t xml:space="preserve">Compliance pattern control</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M4</t>
+          <t xml:space="preserve">Later</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">negotiated_width_o</t>
+          <t xml:space="preserve">txdeemph_o</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DLL sideband / status</t>
+          <t xml:space="preserve">pipe adapter -&gt; PIPE</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">In struct, always 0</t>
+          <t xml:space="preserve">NO (adapter hardcodes 1)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configured Link width after Configuration</t>
+          <t xml:space="preserve">Gen2 de-emphasis selection (-3.5 / -6 dB); negotiated, not constant</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">M4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">negotiated_speed_o</t>
+          <t xml:space="preserve">negotiated_width_o</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -5030,88 +4919,88 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">In struct, always 0</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Current data rate (2.5 GT/s until Recovery.Speed)</t>
+          <t xml:space="preserve">Configured Link width (population count of lane_en)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">active_lane_mask_o</t>
+          <t xml:space="preserve">negotiated_speed_o</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LANES</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_tx / os_rx / DLL</t>
+          <t xml:space="preserve">DLL sideband / status</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO</t>
+          <t xml:space="preserve">Yes (constant 2.5 GT/s)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lanes that form the configured Link</t>
+          <t xml:space="preserve">Current data rate (2.5 GT/s until Recovery.Speed)</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M1 (x2/x4)</t>
+          <t xml:space="preserve">Done (M4)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">accept_dll_tlp_o</t>
+          <t xml:space="preserve">remote_rate_id_o / remote_n_fts_o</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">8 each</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DLL sideband</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">In struct, always 0</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allow DLL traffic (L0 only)</t>
+          <t xml:space="preserve">Peer capability captured in Configuration.Complete, for Recovery.Speed and L0s</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">Done (consumers later)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">replay_freeze_o</t>
+          <t xml:space="preserve">accept_dll_tlp_o</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -5126,47 +5015,79 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">In struct, always 1</t>
+          <t xml:space="preserve">Yes (L0 only)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freeze DLL replay while not in L0</t>
+          <t xml:space="preserve">Allow DLL traffic (L0 only)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">replay_freeze_o</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DLL sideband</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes (inverse of accept_dll_tlp)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freeze DLL replay while not in L0</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">cfg_rx_pm_state_o</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">pipe adapter -&gt; PG239</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">NO (adapter ties 0)</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ASPM RX L0s substate reporting</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Later</t>
         </is>
@@ -5328,7 +5249,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">T_POLLING_ACTIVE_CYC</t>
+          <t xml:space="preserve">T_POLL_ACTIVE_CYC</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -5365,7 +5286,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">T_POLLING_CFG_CYC</t>
+          <t xml:space="preserve">T_POLL_CFG_CYC</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -5698,7 +5619,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N_TS1_MIN</t>
+          <t xml:space="preserve">N_TS1_POLLING</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -5735,7 +5656,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N_TS_CONSEC</t>
+          <t xml:space="preserve">RIVET_N_TS_CONSEC</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -5772,7 +5693,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N_TS2_AFTER_RX</t>
+          <t xml:space="preserve">RIVET_N_TS_AFTER_RX</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -5809,7 +5730,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N_TS1_NUM_CONSEC</t>
+          <t xml:space="preserve">RIVET_N_TS_NUM_CONSEC</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -5846,12 +5767,49 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N_IDLE_RX / N_IDLE_TX</t>
+          <t xml:space="preserve">RIVET_N_IDLE_CONSEC / RIVET_N_IDLE_TX</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">4.2.6.3.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulation divider for every timeout above</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n/a</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">limit / scale</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">limit / scale</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">all timed states</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LTSSM_TIMER_SCALE (rivet_mac / rivet_pcie_ctrl); elaboration checks reject a scale that cannot fit the required TX counts</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
@@ -5864,10 +5822,11 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="78" customWidth="1"/>
-    <col min="4" max="4" width="46" customWidth="1"/>
-    <col min="5" max="5" width="46" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="74" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5883,15 +5842,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Finding</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Where</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Action</t>
         </is>
@@ -5910,17 +5874,22 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rate_o is hardcoded to Gen2 (3'd1). The spec requires 2.5 GT/s for Detect through L0; Polling.Speed is unreachable and Gen2 is reached only via Recovery.Speed.</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">rate_o was hardcoded to Gen2 (3'd1). The spec requires 2.5 GT/s for Detect through L0; Polling.Speed is unreachable and Gen2 is reached only via Recovery.Speed.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">rivet_ltssm.sv</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Drive rate=0 during training; add rate change in M4</t>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rate is 2.5 GT/s; capability advertised in the TS rate ID</t>
         </is>
       </c>
     </row>
@@ -5937,17 +5906,22 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LTSSM has no phystatus / rxelecidle / rx_detected inputs, so it cannot leave Detect for any real reason.</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivet_ltssm.sv ports; rivet_mac_pipe_adapter.sv unused sink</t>
+          <t xml:space="preserve">LTSSM had no phystatus / rxelecidle / rx_detected inputs, so it could not leave Detect for any real reason.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan PHY status out of the adapter into the LTSSM</t>
+          <t xml:space="preserve">rivet_ltssm.sv, rivet_mac_pipe_adapter.sv</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adapter fans PHY status out and decodes RxStatus=011</t>
         </is>
       </c>
     </row>
@@ -5964,17 +5938,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No timers exist and no timer parameters are defined.</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivet_ltssm.sv</t>
+          <t xml:space="preserve">No timers existed and no timer parameters were defined.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add rivet_mac_timer with sim-abbreviated parameters</t>
+          <t xml:space="preserve">rivet_mac_timer.sv, rivet_ltssm.sv</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One shared counter loaded with the limit of the state being entered; LTSSM_TIMER_SCALE shrinks it for simulation</t>
         </is>
       </c>
     </row>
@@ -5991,17 +5970,22 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TS detection is a single link-wide bit with no counting; exits need per-Lane counts (8 consecutive RX, 1024/16 TX).</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">TS detection was a single link-wide bit with no counting; exits need per-Lane counts (8 consecutive RX, 1024/16 TX).</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">rivet_mac_os_rx.sv, rivet_mac_os_tx.sv</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Widen to per-Lane + counters</t>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Per-Lane sliding-window TS detect with per-shape consecutive counters, and a sent counter in os_tx</t>
         </is>
       </c>
     </row>
@@ -6018,17 +6002,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">LinkUp = 1 is set in Configuration.Idle, not on L0 entry.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rivet_ltssm.sv link_up_o</t>
-        </is>
-      </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assert link_up in Config.Idle</t>
+          <t xml:space="preserve">rivet_ltssm.sv</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">link_up asserted in Config.Idle, cleared in Detect.Quiet</t>
         </is>
       </c>
     </row>
@@ -6045,17 +6034,22 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cfg_ltssm_state is not a port on rivet_pcie_ctrl or rivet_pcie; the internal state is consumed by an unused sink.</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivet_pcie_ctrl.sv</t>
+          <t xml:space="preserve">cfg_ltssm_state was not a port on rivet_pcie_ctrl or rivet_pcie; the internal state went to an unused sink.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Expose as PG213-style status output</t>
+          <t xml:space="preserve">rivet_pcie_ctrl.sv, rivet_pcie.sv</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exposed as a PG213-style status output</t>
         </is>
       </c>
     </row>
@@ -6072,17 +6066,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Polling.Configuration must invert Receiver polarity, but rxpolarity is hardcoded to 0 in the adapter.</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Polling.Configuration must invert Receiver polarity, but rxpolarity was hardcoded to 0.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">rivet_mac_pipe_adapter.sv</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Drive from LTSSM / os_rx</t>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Driven from the LTSSM, set from os_rx inversion detect</t>
         </is>
       </c>
     </row>
@@ -6099,17 +6098,22 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configuration.Complete must record the remote data rate identifier and note N_FTS; neither is modelled.</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">os_rx / rivet_ltssm.sv</t>
+          <t xml:space="preserve">Configuration.Complete must record the remote data rate identifier and note N_FTS.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add rate-ID and N_FTS capture (M2)</t>
+          <t xml:space="preserve">rivet_ltssm.sv</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">remote_rate_id / remote_n_fts captured; consumers land with Recovery and L0s</t>
         </is>
       </c>
     </row>
@@ -6126,17 +6130,22 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Lane-to-Lane de-skew must be complete when leaving Config.Complete.</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">rivet_mac_os_rx.sv</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Add deskew_done for x2/x4</t>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deskew_done only checks that every enabled Lane saw a TS in the same cycle; real skew correction is M3</t>
         </is>
       </c>
     </row>
@@ -6153,15 +6162,20 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Enum has no L0s (6'h11-16) or L2 (6'h19-1F) codes, and Loopback naming may not match PG213 exactly.</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">rivet_pkg.sv, docs/mac.md</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirm PG213 table before using those codes</t>
         </is>
@@ -6180,17 +6194,214 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Spec values here come from a local text extract of PCIe Base 2.1; the extract is not redistributable and OCR/layout may be imperfect.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">this workbook</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Verify against the original PDF before RTL sign-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open question</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idle detection counts non-K Symbol Times instead of descrambled 00h, because it is not yet settled whether PG239 scrambles for Gen1/2 or whether the MAC must.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rivet_mac_os_rx.sv, docs/pipe-notes.md</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm scrambler ownership from PG239 / PIPE, then tighten if the MAC sees unscrambled data</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recovery exists only as RcvrLock with a timeout back to Detect, so L0 errors do not actually retrain.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rivet_ltssm.sv</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full Recovery ladder (RcvrLock / RcvrCfg / Idle / Speed) in M4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A partner that configures FEWER Lanes than our port width cannot train: Linkwidth.Start clears link_pad on every enabled Lane instead of narrowing lane_en to the Lanes that received a non-PAD Link number, and Linkwidth.Accept requires a non-PAD Lane number on every enabled Lane. Reproduce with -DRIVET_SMOKE_LANES=4 -DRIVET_SMOKE_PEER_LANES=2 (retrain loop at 6'h06). A partner that is WIDER than us, and Lanes with no Receiver at all, both work.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rivet_ltssm.sv, rivet_mac_os_rx.sv, rivet_mac_os_tx.sv</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M3: per-Lane shape flags out of os_rx, per-Lane PAD control in os_tx, lane_en narrowing in both Linkwidth substates</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lane numbers are always sequential 0..n-1; Lane reversal is not implemented.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rivet_ltssm.sv</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M3 with lane grow</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No scrambler/descrambler exists. Base spec 4.2.3 puts scrambling before 8b/10b encode, and PG239 owns 8b/10b, so this is MAC work. Training is scramble-exempt (K codes plus TS1/TS2 D Symbols), which is why the smoke passes, but Logical Idle is scrambled 00h: against a real Root Port our raw 00h descrambles to garbage, the partner never counts 8 Idle Symbol Times and Configuration.Idle never reaches L0.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rivet_mac_os_tx.sv, rivet_mac_os_rx.sv</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2: per-Lane LFSR G(X)=X^16+X^5+X^4+X^3+1, seed FFFFh, COM re-seeds, SKP does not advance, K and TS bypass, Disable Scrambling bit at end of Config</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No packet datapath through the MAC: dll_tx_ready_o is tied 0 and dll_rx_valid_o tied 0. STP/SDP/END/EDB framing, byte striping across Lanes, real lane-to-lane deskew and L0 SKP scheduling (every 1180-1538 Symbol Times) are all absent.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rivet_mac_os_tx.sv, rivet_mac_os_rx.sv</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 prerequisites before any DLL work</t>
         </is>
       </c>
     </row>

</xml_diff>